<commit_message>
Add dH2_abs_conv/psucc_abs_pref to workbook; guard blank-cell NaN
The two absorption-gate parameters now ship in the Reactions sheet.
dH2_abs_conv is deliberately BLANK because its default is dynamic (it
tracks dH2_conv), which exposed a bug in the code added by bf4bb27: a
blank cell arrives as pandas NaN rather than as an absent key, so
re.get('dH2_abs_conv', dH2_conv) returns NaN and the default never
fires -- float(NaN) then poisons the gate silently.  Use _num(), which
falls back on any non-finite value.  This is the same trap already
documented for loop_net_n_inc / loop_net_w_c.

Verified: with the blank cell, conv_psuccess_abs == conv_psuccess
(2.181172e-06) exactly; with an explicit 0.40 eV it gives 1.344e-01 as
predicted analytically.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/RadCluster_2_1/input/input_parameters.xlsx
+++ b/RadCluster_2_1/input/input_parameters.xlsx
@@ -3108,7 +3108,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E59"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="31.1640625" customWidth="1" style="2" min="1" max="1"/>
@@ -4363,6 +4363,53 @@
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>&lt;100&gt; absorption barrier</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>dH2_abs_conv</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>eV</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Forward barrier for the ABSORPTION success gate P_succ^abs = A_abs*[1+exp((dH2_abs-dH_rev)/kT)]^-1. Blank = dH2_conv (legacy, coupled to junction). Usable 0.30-0.70; junction is 1.00. A &lt;=i_mobile cluster joining a large &lt;100&gt; loop is templated by the host and should not pay the junction reversion penalty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>&lt;100&gt; absorption prefactor</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>psucc_abs_pref</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>1</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>A_abs in P_succ^abs; caps the gate at A_abs/2, so gate&gt;0.5 needs A_abs&gt;1. 1.0 = legacy.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
digital twin calibration runs for eurofer
</commit_message>
<xml_diff>
--- a/RadCluster_2_1/input/input_parameters.xlsx
+++ b/RadCluster_2_1/input/input_parameters.xlsx
@@ -3108,7 +3108,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:E63"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="31.1640625" customWidth="1" style="2" min="1" max="1"/>
@@ -3294,7 +3294,7 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>10000000000000</v>
+        <v>100000000000000</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -3303,7 +3303,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>EUROFER tempered</t>
+          <t>EUROFER97 normalised+tempered martensite. Cold-worked / heavily tempered lath martensite runs 5e14-1e15 m^-2. [2026-08-16: was 1e+13, too low for a tempered-martensitic steel]</t>
         </is>
       </c>
     </row>
@@ -3426,7 +3426,7 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>0.001</v>
+        <v>4e-07</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -3435,7 +3435,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>EUROFER typical</t>
+          <t>EUROFER97 martensite LATH width 0.3-0.5 um.  Was 1e-3 m (1 mm), which gave k2_gb = pi^2/d_g^2 = 9.9e6 m^-2, seven orders below the dislocation sink -- the GB channel was off in all but name.  pi^2/d_g^2 is the lowest slab eigenmode, so lath WIDTH is the right length here.  [2026-08-16: was 0.001]</t>
         </is>
       </c>
     </row>
@@ -3458,7 +3458,7 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>1e+20</v>
+        <v>1e+21</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -3467,7 +3467,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>M23C6 precipitates</t>
+          <t>Effective single population standing in for M23C6 (~1e20 m^-3, r~50 nm) + MX V/Ta carbonitrides (~1e21 m^-3, r~15 nm).  Chosen with r_p=2e-8 to reproduce the COMBINED k2_p = 4*pi*r*rho ~ 2.5e14 m^-2.  [2026-08-16: was 1e+20]</t>
         </is>
       </c>
     </row>
@@ -3483,7 +3483,7 @@
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>5e-08</v>
+        <v>2e-08</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -3492,7 +3492,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>EUROFER typical</t>
+          <t>Effective radius of the combined M23C6+MX population; see rho_p.  [2026-08-16: was 5e-08]</t>
         </is>
       </c>
     </row>
@@ -4407,6 +4407,56 @@
       <c r="E61" t="inlineStr">
         <is>
           <t>A_abs in P_succ^abs; caps the gate at A_abs/2, so gate&gt;0.5 needs A_abs&gt;1. 1.0 = legacy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Lath boundary bias SIA</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Z_gb_i</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Boundary sink bias for SIAs. 1.0 = unbiased = legacy behaviour. Added 2026-08-16: the boundary sink was identical for both species, so it could carry no net bias -- harmless at d_g=1 mm, first-order at the lath width.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Lath boundary bias vac</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Z_gb_v</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>1</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Boundary sink bias for vacancies; paired with Z_gb_i. He is deliberately left unbiased.</t>
         </is>
       </c>
     </row>

</xml_diff>